<commit_message>
fix excel template f3
</commit_message>
<xml_diff>
--- a/Bath_Image.xlsx
+++ b/Bath_Image.xlsx
@@ -554,7 +554,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="46.5" customHeight="1">
+    <row r="2" ht="19.5" customHeight="1">
       <c r="A2" s="7" t="inlineStr">
         <is>
           <t>IATE</t>
@@ -562,12 +562,12 @@
       </c>
       <c r="B2" s="7" t="inlineStr">
         <is>
-          <t>Dog</t>
+          <t>Rabit</t>
         </is>
       </c>
       <c r="C2" s="7" t="inlineStr">
         <is>
-          <t>C:\Users\Admin\Downloads\Auto_download_mockup\Image_src\I've appeared that' enough\Dog.png</t>
+          <t>C:\Users\Admin\Downloads\Auto_download_mockup\Image_src\I've appeared that' enough\Rabit.png</t>
         </is>
       </c>
       <c r="D2" s="8" t="inlineStr">
@@ -582,37 +582,17 @@
       </c>
       <c r="F2" s="7" t="inlineStr">
         <is>
-          <t>OK | 16 ảnh | customG_0=tcndscb363 | C:\Users\Admin\Downloads\Auto_download_mockup\Image_src\I've appeared that' enough\IATE-Dog</t>
+          <t>OK | 16 ảnh | customG_0=tcyckw09e6 | C:\Users\Admin\Downloads\Auto_download_mockup\Image_src\I've appeared that' enough\IATE-Rab</t>
         </is>
       </c>
     </row>
     <row r="3" ht="19.5" customHeight="1">
-      <c r="A3" s="7" t="inlineStr">
-        <is>
-          <t>IATE</t>
-        </is>
-      </c>
-      <c r="B3" s="7" t="inlineStr">
-        <is>
-          <t>Cat</t>
-        </is>
-      </c>
-      <c r="C3" s="7" t="inlineStr">
-        <is>
-          <t>C:\Users\Admin\Downloads\Auto_download_mockup\Image_src\I've appeared that' enough\Cat.png</t>
-        </is>
-      </c>
-      <c r="D3" s="9" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="E3" s="9" t="inlineStr">
-        <is>
-          <t>Running</t>
-        </is>
-      </c>
-      <c r="F3" s="4" t="inlineStr"/>
+      <c r="A3" s="7" t="n"/>
+      <c r="B3" s="7" t="n"/>
+      <c r="C3" s="7" t="n"/>
+      <c r="D3" s="9" t="n"/>
+      <c r="E3" s="9" t="n"/>
+      <c r="F3" s="4" t="n"/>
     </row>
     <row r="4" ht="19.5" customHeight="1">
       <c r="A4" s="4" t="n"/>

</xml_diff>

<commit_message>
update gen file template
</commit_message>
<xml_diff>
--- a/Bath_Image.xlsx
+++ b/Bath_Image.xlsx
@@ -111,7 +111,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
@@ -136,6 +136,12 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="1" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="1" xfId="0">
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -514,12 +520,12 @@
   <dimension ref="A1:F30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
-    <col width="18.005" bestFit="1" customWidth="1" style="10" min="1" max="1"/>
-    <col width="22.005" bestFit="1" customWidth="1" style="10" min="2" max="2"/>
-    <col width="101.005" bestFit="1" customWidth="1" style="10" min="3" max="3"/>
-    <col width="12.005" bestFit="1" customWidth="1" style="11" min="4" max="4"/>
-    <col width="14.005" bestFit="1" customWidth="1" style="11" min="5" max="5"/>
-    <col width="34.005" bestFit="1" customWidth="1" style="10" min="6" max="6"/>
+    <col width="18.005" bestFit="1" customWidth="1" style="12" min="1" max="1"/>
+    <col width="22.005" bestFit="1" customWidth="1" style="12" min="2" max="2"/>
+    <col width="101.005" bestFit="1" customWidth="1" style="12" min="3" max="3"/>
+    <col width="12.005" bestFit="1" customWidth="1" style="13" min="4" max="4"/>
+    <col width="14.005" bestFit="1" customWidth="1" style="13" min="5" max="5"/>
+    <col width="34.005" bestFit="1" customWidth="1" style="12" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -567,7 +573,7 @@
       </c>
       <c r="C2" s="7" t="inlineStr">
         <is>
-          <t>C:\Users\Admin\Downloads\Auto_download_mockup\Image_src\I've appeared that' enough\Rabit.png</t>
+          <t>C:\Users\Admin\Downloads\Auto_download_mockup\Image_src\I've appeared that' enough\abit.png</t>
         </is>
       </c>
       <c r="D2" s="8" t="inlineStr">
@@ -575,14 +581,14 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="E2" s="8" t="inlineStr">
+      <c r="E2" s="9" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="F2" s="7" t="inlineStr">
-        <is>
-          <t>OK | 16 ảnh | customG_0=tcyckw09e6 | C:\Users\Admin\Downloads\Auto_download_mockup\Image_src\I've appeared that' enough\IATE-Rab</t>
+      <c r="F2" s="10" t="inlineStr">
+        <is>
+          <t>OK | 8 ảnh | customG_0=tcz6al6549 | C:\Users\Admin\Downloads\Auto_download_mockup\Image_src\I've appeared that' enough\IATE-abi</t>
         </is>
       </c>
     </row>
@@ -590,224 +596,224 @@
       <c r="A3" s="7" t="n"/>
       <c r="B3" s="7" t="n"/>
       <c r="C3" s="7" t="n"/>
-      <c r="D3" s="9" t="n"/>
-      <c r="E3" s="9" t="n"/>
+      <c r="D3" s="11" t="n"/>
+      <c r="E3" s="11" t="n"/>
       <c r="F3" s="4" t="n"/>
     </row>
     <row r="4" ht="19.5" customHeight="1">
       <c r="A4" s="4" t="n"/>
       <c r="B4" s="4" t="n"/>
       <c r="C4" s="4" t="n"/>
-      <c r="D4" s="9" t="n"/>
-      <c r="E4" s="9" t="n"/>
+      <c r="D4" s="11" t="n"/>
+      <c r="E4" s="11" t="n"/>
       <c r="F4" s="4" t="n"/>
     </row>
     <row r="5" ht="19.5" customHeight="1">
       <c r="A5" s="4" t="n"/>
       <c r="B5" s="4" t="n"/>
       <c r="C5" s="4" t="n"/>
-      <c r="D5" s="9" t="n"/>
-      <c r="E5" s="9" t="n"/>
+      <c r="D5" s="11" t="n"/>
+      <c r="E5" s="11" t="n"/>
       <c r="F5" s="4" t="n"/>
     </row>
     <row r="6" ht="19.5" customHeight="1">
       <c r="A6" s="4" t="n"/>
       <c r="B6" s="4" t="n"/>
       <c r="C6" s="4" t="n"/>
-      <c r="D6" s="9" t="n"/>
-      <c r="E6" s="9" t="n"/>
+      <c r="D6" s="11" t="n"/>
+      <c r="E6" s="11" t="n"/>
       <c r="F6" s="4" t="n"/>
     </row>
     <row r="7" ht="19.5" customHeight="1">
       <c r="A7" s="4" t="n"/>
       <c r="B7" s="4" t="n"/>
       <c r="C7" s="4" t="n"/>
-      <c r="D7" s="9" t="n"/>
-      <c r="E7" s="9" t="n"/>
+      <c r="D7" s="11" t="n"/>
+      <c r="E7" s="11" t="n"/>
       <c r="F7" s="4" t="n"/>
     </row>
     <row r="8" ht="19.5" customHeight="1">
       <c r="A8" s="4" t="n"/>
       <c r="B8" s="4" t="n"/>
       <c r="C8" s="4" t="n"/>
-      <c r="D8" s="9" t="n"/>
-      <c r="E8" s="9" t="n"/>
+      <c r="D8" s="11" t="n"/>
+      <c r="E8" s="11" t="n"/>
       <c r="F8" s="4" t="n"/>
     </row>
     <row r="9" ht="19.5" customHeight="1">
       <c r="A9" s="4" t="n"/>
       <c r="B9" s="4" t="n"/>
       <c r="C9" s="4" t="n"/>
-      <c r="D9" s="9" t="n"/>
-      <c r="E9" s="9" t="n"/>
+      <c r="D9" s="11" t="n"/>
+      <c r="E9" s="11" t="n"/>
       <c r="F9" s="4" t="n"/>
     </row>
     <row r="10" ht="19.5" customHeight="1">
       <c r="A10" s="4" t="n"/>
       <c r="B10" s="4" t="n"/>
       <c r="C10" s="4" t="n"/>
-      <c r="D10" s="9" t="n"/>
-      <c r="E10" s="9" t="n"/>
+      <c r="D10" s="11" t="n"/>
+      <c r="E10" s="11" t="n"/>
       <c r="F10" s="4" t="n"/>
     </row>
     <row r="11" ht="19.5" customHeight="1">
       <c r="A11" s="4" t="n"/>
       <c r="B11" s="4" t="n"/>
       <c r="C11" s="4" t="n"/>
-      <c r="D11" s="9" t="n"/>
-      <c r="E11" s="9" t="n"/>
+      <c r="D11" s="11" t="n"/>
+      <c r="E11" s="11" t="n"/>
       <c r="F11" s="4" t="n"/>
     </row>
     <row r="12" ht="19.5" customHeight="1">
       <c r="A12" s="4" t="n"/>
       <c r="B12" s="4" t="n"/>
       <c r="C12" s="4" t="n"/>
-      <c r="D12" s="9" t="n"/>
-      <c r="E12" s="9" t="n"/>
+      <c r="D12" s="11" t="n"/>
+      <c r="E12" s="11" t="n"/>
       <c r="F12" s="4" t="n"/>
     </row>
     <row r="13" ht="19.5" customHeight="1">
       <c r="A13" s="4" t="n"/>
       <c r="B13" s="4" t="n"/>
       <c r="C13" s="4" t="n"/>
-      <c r="D13" s="9" t="n"/>
-      <c r="E13" s="9" t="n"/>
+      <c r="D13" s="11" t="n"/>
+      <c r="E13" s="11" t="n"/>
       <c r="F13" s="4" t="n"/>
     </row>
     <row r="14" ht="19.5" customHeight="1">
       <c r="A14" s="4" t="n"/>
       <c r="B14" s="4" t="n"/>
       <c r="C14" s="4" t="n"/>
-      <c r="D14" s="9" t="n"/>
-      <c r="E14" s="9" t="n"/>
+      <c r="D14" s="11" t="n"/>
+      <c r="E14" s="11" t="n"/>
       <c r="F14" s="4" t="n"/>
     </row>
     <row r="15" ht="19.5" customHeight="1">
       <c r="A15" s="4" t="n"/>
       <c r="B15" s="4" t="n"/>
       <c r="C15" s="4" t="n"/>
-      <c r="D15" s="9" t="n"/>
-      <c r="E15" s="9" t="n"/>
+      <c r="D15" s="11" t="n"/>
+      <c r="E15" s="11" t="n"/>
       <c r="F15" s="4" t="n"/>
     </row>
     <row r="16" ht="19.5" customHeight="1">
       <c r="A16" s="4" t="n"/>
       <c r="B16" s="4" t="n"/>
       <c r="C16" s="4" t="n"/>
-      <c r="D16" s="9" t="n"/>
-      <c r="E16" s="9" t="n"/>
+      <c r="D16" s="11" t="n"/>
+      <c r="E16" s="11" t="n"/>
       <c r="F16" s="4" t="n"/>
     </row>
     <row r="17" ht="19.5" customHeight="1">
       <c r="A17" s="4" t="n"/>
       <c r="B17" s="4" t="n"/>
       <c r="C17" s="4" t="n"/>
-      <c r="D17" s="9" t="n"/>
-      <c r="E17" s="9" t="n"/>
+      <c r="D17" s="11" t="n"/>
+      <c r="E17" s="11" t="n"/>
       <c r="F17" s="4" t="n"/>
     </row>
     <row r="18" ht="19.5" customHeight="1">
       <c r="A18" s="4" t="n"/>
       <c r="B18" s="4" t="n"/>
       <c r="C18" s="4" t="n"/>
-      <c r="D18" s="9" t="n"/>
-      <c r="E18" s="9" t="n"/>
+      <c r="D18" s="11" t="n"/>
+      <c r="E18" s="11" t="n"/>
       <c r="F18" s="4" t="n"/>
     </row>
     <row r="19" ht="19.5" customHeight="1">
       <c r="A19" s="4" t="n"/>
       <c r="B19" s="4" t="n"/>
       <c r="C19" s="4" t="n"/>
-      <c r="D19" s="9" t="n"/>
-      <c r="E19" s="9" t="n"/>
+      <c r="D19" s="11" t="n"/>
+      <c r="E19" s="11" t="n"/>
       <c r="F19" s="4" t="n"/>
     </row>
     <row r="20" ht="19.5" customHeight="1">
       <c r="A20" s="4" t="n"/>
       <c r="B20" s="4" t="n"/>
       <c r="C20" s="4" t="n"/>
-      <c r="D20" s="9" t="n"/>
-      <c r="E20" s="9" t="n"/>
+      <c r="D20" s="11" t="n"/>
+      <c r="E20" s="11" t="n"/>
       <c r="F20" s="4" t="n"/>
     </row>
     <row r="21" ht="19.5" customHeight="1">
       <c r="A21" s="4" t="n"/>
       <c r="B21" s="4" t="n"/>
       <c r="C21" s="4" t="n"/>
-      <c r="D21" s="9" t="n"/>
-      <c r="E21" s="9" t="n"/>
+      <c r="D21" s="11" t="n"/>
+      <c r="E21" s="11" t="n"/>
       <c r="F21" s="4" t="n"/>
     </row>
     <row r="22" ht="19.5" customHeight="1">
       <c r="A22" s="4" t="n"/>
       <c r="B22" s="4" t="n"/>
       <c r="C22" s="4" t="n"/>
-      <c r="D22" s="9" t="n"/>
-      <c r="E22" s="9" t="n"/>
+      <c r="D22" s="11" t="n"/>
+      <c r="E22" s="11" t="n"/>
       <c r="F22" s="4" t="n"/>
     </row>
     <row r="23" ht="19.5" customHeight="1">
       <c r="A23" s="4" t="n"/>
       <c r="B23" s="4" t="n"/>
       <c r="C23" s="4" t="n"/>
-      <c r="D23" s="9" t="n"/>
-      <c r="E23" s="9" t="n"/>
+      <c r="D23" s="11" t="n"/>
+      <c r="E23" s="11" t="n"/>
       <c r="F23" s="4" t="n"/>
     </row>
     <row r="24" ht="18.75" customHeight="1">
       <c r="A24" s="4" t="n"/>
       <c r="B24" s="4" t="n"/>
       <c r="C24" s="4" t="n"/>
-      <c r="D24" s="9" t="n"/>
-      <c r="E24" s="9" t="n"/>
+      <c r="D24" s="11" t="n"/>
+      <c r="E24" s="11" t="n"/>
       <c r="F24" s="4" t="n"/>
     </row>
     <row r="25" ht="18.75" customHeight="1">
       <c r="A25" s="4" t="n"/>
       <c r="B25" s="4" t="n"/>
       <c r="C25" s="4" t="n"/>
-      <c r="D25" s="9" t="n"/>
-      <c r="E25" s="9" t="n"/>
+      <c r="D25" s="11" t="n"/>
+      <c r="E25" s="11" t="n"/>
       <c r="F25" s="4" t="n"/>
     </row>
     <row r="26" ht="18.75" customHeight="1">
       <c r="A26" s="4" t="n"/>
       <c r="B26" s="4" t="n"/>
       <c r="C26" s="4" t="n"/>
-      <c r="D26" s="9" t="n"/>
-      <c r="E26" s="9" t="n"/>
+      <c r="D26" s="11" t="n"/>
+      <c r="E26" s="11" t="n"/>
       <c r="F26" s="4" t="n"/>
     </row>
     <row r="27" ht="18.75" customHeight="1">
       <c r="A27" s="4" t="n"/>
       <c r="B27" s="4" t="n"/>
       <c r="C27" s="4" t="n"/>
-      <c r="D27" s="9" t="n"/>
-      <c r="E27" s="9" t="n"/>
+      <c r="D27" s="11" t="n"/>
+      <c r="E27" s="11" t="n"/>
       <c r="F27" s="4" t="n"/>
     </row>
     <row r="28" ht="18.75" customHeight="1">
       <c r="A28" s="4" t="n"/>
       <c r="B28" s="4" t="n"/>
       <c r="C28" s="4" t="n"/>
-      <c r="D28" s="9" t="n"/>
-      <c r="E28" s="9" t="n"/>
+      <c r="D28" s="11" t="n"/>
+      <c r="E28" s="11" t="n"/>
       <c r="F28" s="4" t="n"/>
     </row>
     <row r="29" ht="18.75" customHeight="1">
       <c r="A29" s="4" t="n"/>
       <c r="B29" s="4" t="n"/>
       <c r="C29" s="4" t="n"/>
-      <c r="D29" s="9" t="n"/>
-      <c r="E29" s="9" t="n"/>
+      <c r="D29" s="11" t="n"/>
+      <c r="E29" s="11" t="n"/>
       <c r="F29" s="4" t="n"/>
     </row>
     <row r="30" ht="18.75" customHeight="1">
       <c r="A30" s="4" t="n"/>
       <c r="B30" s="4" t="n"/>
       <c r="C30" s="4" t="n"/>
-      <c r="D30" s="9" t="n"/>
-      <c r="E30" s="9" t="n"/>
+      <c r="D30" s="11" t="n"/>
+      <c r="E30" s="11" t="n"/>
       <c r="F30" s="4" t="n"/>
     </row>
   </sheetData>

</xml_diff>